<commit_message>
Feature/add new functiosn (#15)
* add changes

* add new endpoint json

* add class-validator/class-transformer

* add mejoras

* add upload drive
</commit_message>
<xml_diff>
--- a/src/data/input/business_actors.xlsx
+++ b/src/data/input/business_actors.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Files\Github\back-dinamic-architect\src\data\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AntonioAlonsoPerez\Documents\Github\back-dinamic-architect\src\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F16380-38E9-43E3-80DB-317FE8FF4DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02DD8401-62C5-4FA5-B3F4-1C9E5F2DD033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6E292256-CBF0-9F4E-B151-1D63BF0EB61C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{6E292256-CBF0-9F4E-B151-1D63BF0EB61C}"/>
   </bookViews>
   <sheets>
     <sheet name="BusinessActors" sheetId="1" r:id="rId1"/>
-    <sheet name="Drivers" sheetId="2" r:id="rId2"/>
-    <sheet name="Goals" sheetId="3" r:id="rId3"/>
-    <sheet name="Results" sheetId="4" r:id="rId4"/>
-    <sheet name="Plan" sheetId="5" r:id="rId5"/>
+    <sheet name="Driver" sheetId="2" r:id="rId2"/>
+    <sheet name="Goal" sheetId="3" r:id="rId3"/>
+    <sheet name="Principle" sheetId="4" r:id="rId4"/>
+    <sheet name="CourseOfAction" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>name</t>
   </si>
@@ -54,32 +54,44 @@
     <t>Drivers</t>
   </si>
   <si>
-    <t>Incrementar la cartera de Macropay integrando prestamos desde la aplicación</t>
-  </si>
-  <si>
     <t>Goals</t>
   </si>
   <si>
-    <t>Mejorar la experiencia del cliente de manera eficiente y efectiva</t>
-  </si>
-  <si>
     <t>Results</t>
   </si>
   <si>
-    <t>Implementar la adquisición de préstamos desde la aplicación de Macropay</t>
-  </si>
-  <si>
-    <t>Plan</t>
-  </si>
-  <si>
-    <t>Brindar un flujo denominado Prestamos gestionado desde la App Macropay</t>
+    <t>texto resultados</t>
+  </si>
+  <si>
+    <t>texto goal</t>
+  </si>
+  <si>
+    <t>texto driver</t>
+  </si>
+  <si>
+    <t>texto plan</t>
+  </si>
+  <si>
+    <t>Aplicaciones</t>
+  </si>
+  <si>
+    <t>texto driver 2</t>
+  </si>
+  <si>
+    <t>texto goal 2</t>
+  </si>
+  <si>
+    <t>texto resultados 2</t>
+  </si>
+  <si>
+    <t>texto plan 2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -97,6 +109,12 @@
       <u/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -460,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9862910F-884A-0146-8552-537FA771751A}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -478,6 +496,11 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -485,7 +508,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA1B24C8-BC7C-46BB-9838-57445A49E5D4}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="65" bestFit="1" customWidth="1"/>
@@ -498,7 +521,12 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -516,12 +544,17 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -538,7 +571,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B69CE35B-DD04-48D4-B659-46A893DCE43C}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="62.375" bestFit="1" customWidth="1"/>
@@ -546,12 +579,17 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -574,10 +612,11 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>